<commit_message>
Generate Excel reports automatically inside E2E and K6 actions
</commit_message>
<xml_diff>
--- a/k6_load_test_report.xlsx
+++ b/k6_load_test_report.xlsx
@@ -570,8 +570,8 @@
         <is>
           <t>PERFORMANCE STATUS: PASSED
 - All API and Frontend request thresholds satisfied.
-- Average response latency is under 50ms.
-- Zero HTTP connection errors detected.
+- Success rate: 100.0%
+- 95% latency: 92.5 ms
 - Deployable for staging validation.</t>
         </is>
       </c>
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>39</v>
+        <v>93</v>
       </c>
       <c r="F2" s="9" t="n">
         <v>200</v>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>200</v>
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>200</v>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>200</v>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>50</v>
+        <v>88</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>200</v>
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>200</v>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>200</v>
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>200</v>
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>200</v>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>200</v>
@@ -1096,7 +1096,7 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="F12" s="9" t="n">
         <v>200</v>
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>200</v>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F14" s="9" t="n">
         <v>200</v>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>200</v>
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="F16" s="9" t="n">
         <v>200</v>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>200</v>
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="F18" s="9" t="n">
         <v>200</v>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>200</v>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="F20" s="9" t="n">
         <v>200</v>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>200</v>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F22" s="9" t="n">
         <v>200</v>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>200</v>
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="F24" s="9" t="n">
         <v>200</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>37</v>
+        <v>92</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>200</v>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>200</v>
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>200</v>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F28" s="9" t="n">
         <v>200</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>200</v>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>200</v>
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>200</v>
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>10</v>
+        <v>85</v>
       </c>
       <c r="F32" s="9" t="n">
         <v>200</v>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>200</v>
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F34" s="9" t="n">
         <v>200</v>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>200</v>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="F36" s="9" t="n">
         <v>200</v>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>200</v>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>200</v>
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="F39" s="9" t="n">
         <v>200</v>
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="E40" s="5" t="n">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="F40" s="9" t="n">
         <v>200</v>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>200</v>
@@ -2086,7 +2086,7 @@
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="F42" s="9" t="n">
         <v>200</v>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="E43" s="5" t="n">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="F43" s="9" t="n">
         <v>200</v>
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>200</v>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="F45" s="9" t="n">
         <v>200</v>
@@ -2218,7 +2218,7 @@
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F46" s="9" t="n">
         <v>200</v>
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F47" s="9" t="n">
         <v>200</v>
@@ -2284,7 +2284,7 @@
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="F48" s="9" t="n">
         <v>200</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="F49" s="9" t="n">
         <v>200</v>
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="F50" s="9" t="n">
         <v>200</v>
@@ -2383,7 +2383,7 @@
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F51" s="9" t="n">
         <v>200</v>
@@ -2416,7 +2416,7 @@
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="F52" s="9" t="n">
         <v>200</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="F53" s="9" t="n">
         <v>200</v>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="F54" s="9" t="n">
         <v>200</v>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="F55" s="9" t="n">
         <v>200</v>
@@ -2548,7 +2548,7 @@
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="F56" s="9" t="n">
         <v>200</v>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="F57" s="9" t="n">
         <v>200</v>
@@ -2614,7 +2614,7 @@
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="F58" s="9" t="n">
         <v>200</v>
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="F59" s="9" t="n">
         <v>200</v>
@@ -2680,7 +2680,7 @@
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="F60" s="9" t="n">
         <v>200</v>
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F61" s="9" t="n">
         <v>200</v>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="F62" s="9" t="n">
         <v>200</v>
@@ -2779,7 +2779,7 @@
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="F63" s="9" t="n">
         <v>200</v>
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="E64" s="5" t="n">
-        <v>89</v>
+        <v>15</v>
       </c>
       <c r="F64" s="9" t="n">
         <v>200</v>
@@ -2845,7 +2845,7 @@
         </is>
       </c>
       <c r="E65" s="5" t="n">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="F65" s="9" t="n">
         <v>200</v>
@@ -2878,7 +2878,7 @@
         </is>
       </c>
       <c r="E66" s="5" t="n">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="F66" s="9" t="n">
         <v>200</v>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="E67" s="5" t="n">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="F67" s="9" t="n">
         <v>200</v>
@@ -2944,7 +2944,7 @@
         </is>
       </c>
       <c r="E68" s="5" t="n">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="F68" s="9" t="n">
         <v>200</v>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="E69" s="5" t="n">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="F69" s="9" t="n">
         <v>200</v>
@@ -3010,7 +3010,7 @@
         </is>
       </c>
       <c r="E70" s="5" t="n">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="F70" s="9" t="n">
         <v>200</v>
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="E72" s="5" t="n">
-        <v>86</v>
+        <v>47</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>200</v>
@@ -3109,7 +3109,7 @@
         </is>
       </c>
       <c r="E73" s="5" t="n">
-        <v>51</v>
+        <v>94</v>
       </c>
       <c r="F73" s="9" t="n">
         <v>200</v>
@@ -3142,7 +3142,7 @@
         </is>
       </c>
       <c r="E74" s="5" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="F74" s="9" t="n">
         <v>200</v>
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="E75" s="5" t="n">
-        <v>26</v>
+        <v>69</v>
       </c>
       <c r="F75" s="9" t="n">
         <v>200</v>
@@ -3208,7 +3208,7 @@
         </is>
       </c>
       <c r="E76" s="5" t="n">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="F76" s="9" t="n">
         <v>200</v>
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="E77" s="5" t="n">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="F77" s="9" t="n">
         <v>200</v>
@@ -3274,7 +3274,7 @@
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="F78" s="9" t="n">
         <v>200</v>
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="E79" s="5" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="F79" s="9" t="n">
         <v>200</v>
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="E80" s="5" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="F80" s="9" t="n">
         <v>200</v>
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="E81" s="5" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="F81" s="9" t="n">
         <v>200</v>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="E82" s="5" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F82" s="9" t="n">
         <v>200</v>
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="E83" s="5" t="n">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="F83" s="9" t="n">
         <v>200</v>
@@ -3472,7 +3472,7 @@
         </is>
       </c>
       <c r="E84" s="5" t="n">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="F84" s="9" t="n">
         <v>200</v>
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="E85" s="5" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F85" s="9" t="n">
         <v>200</v>
@@ -3538,7 +3538,7 @@
         </is>
       </c>
       <c r="E86" s="5" t="n">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="F86" s="9" t="n">
         <v>200</v>
@@ -3571,7 +3571,7 @@
         </is>
       </c>
       <c r="E87" s="5" t="n">
-        <v>53</v>
+        <v>93</v>
       </c>
       <c r="F87" s="9" t="n">
         <v>200</v>
@@ -3604,7 +3604,7 @@
         </is>
       </c>
       <c r="E88" s="5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F88" s="9" t="n">
         <v>200</v>
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="E89" s="5" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="F89" s="9" t="n">
         <v>200</v>
@@ -3670,7 +3670,7 @@
         </is>
       </c>
       <c r="E90" s="5" t="n">
-        <v>82</v>
+        <v>17</v>
       </c>
       <c r="F90" s="9" t="n">
         <v>200</v>
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="E91" s="5" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="F91" s="9" t="n">
         <v>200</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="E92" s="5" t="n">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="F92" s="9" t="n">
         <v>200</v>
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="E93" s="5" t="n">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="F93" s="9" t="n">
         <v>200</v>
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="E94" s="5" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F94" s="9" t="n">
         <v>200</v>
@@ -3835,7 +3835,7 @@
         </is>
       </c>
       <c r="E95" s="5" t="n">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="F95" s="9" t="n">
         <v>200</v>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="E96" s="5" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F96" s="9" t="n">
         <v>200</v>
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="E97" s="5" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F97" s="9" t="n">
         <v>200</v>
@@ -3934,7 +3934,7 @@
         </is>
       </c>
       <c r="E98" s="5" t="n">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="F98" s="9" t="n">
         <v>200</v>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="E99" s="5" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="F99" s="9" t="n">
         <v>200</v>
@@ -4000,7 +4000,7 @@
         </is>
       </c>
       <c r="E100" s="5" t="n">
-        <v>26</v>
+        <v>73</v>
       </c>
       <c r="F100" s="9" t="n">
         <v>200</v>
@@ -4033,7 +4033,7 @@
         </is>
       </c>
       <c r="E101" s="5" t="n">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="F101" s="9" t="n">
         <v>200</v>
@@ -4066,7 +4066,7 @@
         </is>
       </c>
       <c r="E102" s="5" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="F102" s="9" t="n">
         <v>200</v>
@@ -4099,7 +4099,7 @@
         </is>
       </c>
       <c r="E103" s="5" t="n">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="F103" s="9" t="n">
         <v>200</v>
@@ -4132,7 +4132,7 @@
         </is>
       </c>
       <c r="E104" s="5" t="n">
-        <v>16</v>
+        <v>73</v>
       </c>
       <c r="F104" s="9" t="n">
         <v>200</v>
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="E105" s="5" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="F105" s="9" t="n">
         <v>200</v>
@@ -4198,7 +4198,7 @@
         </is>
       </c>
       <c r="E106" s="5" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="F106" s="9" t="n">
         <v>200</v>
@@ -4231,7 +4231,7 @@
         </is>
       </c>
       <c r="E107" s="5" t="n">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="F107" s="9" t="n">
         <v>200</v>
@@ -4264,7 +4264,7 @@
         </is>
       </c>
       <c r="E108" s="5" t="n">
-        <v>27</v>
+        <v>67</v>
       </c>
       <c r="F108" s="9" t="n">
         <v>200</v>
@@ -4297,7 +4297,7 @@
         </is>
       </c>
       <c r="E109" s="5" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="F109" s="9" t="n">
         <v>200</v>
@@ -4330,7 +4330,7 @@
         </is>
       </c>
       <c r="E110" s="5" t="n">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="F110" s="9" t="n">
         <v>200</v>
@@ -4363,7 +4363,7 @@
         </is>
       </c>
       <c r="E111" s="5" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="F111" s="9" t="n">
         <v>200</v>
@@ -4396,7 +4396,7 @@
         </is>
       </c>
       <c r="E112" s="5" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="F112" s="9" t="n">
         <v>200</v>
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="E113" s="5" t="n">
-        <v>54</v>
+        <v>84</v>
       </c>
       <c r="F113" s="9" t="n">
         <v>200</v>
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="E114" s="5" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F114" s="9" t="n">
         <v>200</v>
@@ -4495,7 +4495,7 @@
         </is>
       </c>
       <c r="E115" s="5" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F115" s="9" t="n">
         <v>200</v>
@@ -4528,7 +4528,7 @@
         </is>
       </c>
       <c r="E116" s="5" t="n">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="F116" s="9" t="n">
         <v>200</v>
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="E117" s="5" t="n">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="F117" s="9" t="n">
         <v>200</v>
@@ -4594,7 +4594,7 @@
         </is>
       </c>
       <c r="E118" s="5" t="n">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="F118" s="9" t="n">
         <v>200</v>
@@ -4627,7 +4627,7 @@
         </is>
       </c>
       <c r="E119" s="5" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="F119" s="9" t="n">
         <v>200</v>
@@ -4660,7 +4660,7 @@
         </is>
       </c>
       <c r="E120" s="5" t="n">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="F120" s="9" t="n">
         <v>200</v>
@@ -4693,7 +4693,7 @@
         </is>
       </c>
       <c r="E121" s="5" t="n">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="F121" s="9" t="n">
         <v>200</v>
@@ -4726,7 +4726,7 @@
         </is>
       </c>
       <c r="E122" s="5" t="n">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="F122" s="9" t="n">
         <v>200</v>
@@ -4759,7 +4759,7 @@
         </is>
       </c>
       <c r="E123" s="5" t="n">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="F123" s="9" t="n">
         <v>200</v>
@@ -4792,7 +4792,7 @@
         </is>
       </c>
       <c r="E124" s="5" t="n">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="F124" s="9" t="n">
         <v>200</v>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="E125" s="5" t="n">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="F125" s="9" t="n">
         <v>200</v>
@@ -4858,7 +4858,7 @@
         </is>
       </c>
       <c r="E126" s="5" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="F126" s="9" t="n">
         <v>200</v>
@@ -4891,7 +4891,7 @@
         </is>
       </c>
       <c r="E127" s="5" t="n">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="F127" s="9" t="n">
         <v>200</v>
@@ -4924,7 +4924,7 @@
         </is>
       </c>
       <c r="E128" s="5" t="n">
-        <v>63</v>
+        <v>93</v>
       </c>
       <c r="F128" s="9" t="n">
         <v>200</v>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="E129" s="5" t="n">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="F129" s="9" t="n">
         <v>200</v>
@@ -4990,7 +4990,7 @@
         </is>
       </c>
       <c r="E130" s="5" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="F130" s="9" t="n">
         <v>200</v>
@@ -5023,7 +5023,7 @@
         </is>
       </c>
       <c r="E131" s="5" t="n">
-        <v>57</v>
+        <v>85</v>
       </c>
       <c r="F131" s="9" t="n">
         <v>200</v>
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="E132" s="5" t="n">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="F132" s="9" t="n">
         <v>200</v>
@@ -5089,7 +5089,7 @@
         </is>
       </c>
       <c r="E133" s="5" t="n">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="F133" s="9" t="n">
         <v>200</v>
@@ -5122,7 +5122,7 @@
         </is>
       </c>
       <c r="E134" s="5" t="n">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="F134" s="9" t="n">
         <v>200</v>
@@ -5155,7 +5155,7 @@
         </is>
       </c>
       <c r="E135" s="5" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="F135" s="9" t="n">
         <v>200</v>
@@ -5188,7 +5188,7 @@
         </is>
       </c>
       <c r="E136" s="5" t="n">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="F136" s="9" t="n">
         <v>200</v>
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="E137" s="5" t="n">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="F137" s="9" t="n">
         <v>200</v>
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="E138" s="5" t="n">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="F138" s="9" t="n">
         <v>200</v>
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="E139" s="5" t="n">
-        <v>21</v>
+        <v>94</v>
       </c>
       <c r="F139" s="9" t="n">
         <v>200</v>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="E141" s="5" t="n">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="F141" s="9" t="n">
         <v>200</v>
@@ -5386,7 +5386,7 @@
         </is>
       </c>
       <c r="E142" s="5" t="n">
-        <v>94</v>
+        <v>65</v>
       </c>
       <c r="F142" s="9" t="n">
         <v>200</v>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="E143" s="5" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F143" s="9" t="n">
         <v>200</v>
@@ -5452,7 +5452,7 @@
         </is>
       </c>
       <c r="E144" s="5" t="n">
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="F144" s="9" t="n">
         <v>200</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="E145" s="5" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="F145" s="9" t="n">
         <v>200</v>
@@ -5518,7 +5518,7 @@
         </is>
       </c>
       <c r="E146" s="5" t="n">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="F146" s="9" t="n">
         <v>200</v>
@@ -5551,7 +5551,7 @@
         </is>
       </c>
       <c r="E147" s="5" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="F147" s="9" t="n">
         <v>200</v>
@@ -5584,7 +5584,7 @@
         </is>
       </c>
       <c r="E148" s="5" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F148" s="9" t="n">
         <v>200</v>
@@ -5617,7 +5617,7 @@
         </is>
       </c>
       <c r="E149" s="5" t="n">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="F149" s="9" t="n">
         <v>200</v>
@@ -5650,7 +5650,7 @@
         </is>
       </c>
       <c r="E150" s="5" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F150" s="9" t="n">
         <v>200</v>
@@ -5683,7 +5683,7 @@
         </is>
       </c>
       <c r="E151" s="5" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F151" s="9" t="n">
         <v>200</v>
@@ -5749,7 +5749,7 @@
         </is>
       </c>
       <c r="E153" s="5" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="F153" s="9" t="n">
         <v>200</v>
@@ -5782,7 +5782,7 @@
         </is>
       </c>
       <c r="E154" s="5" t="n">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="F154" s="9" t="n">
         <v>200</v>
@@ -5815,7 +5815,7 @@
         </is>
       </c>
       <c r="E155" s="5" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="F155" s="9" t="n">
         <v>200</v>
@@ -5848,7 +5848,7 @@
         </is>
       </c>
       <c r="E156" s="5" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="F156" s="9" t="n">
         <v>200</v>
@@ -5881,7 +5881,7 @@
         </is>
       </c>
       <c r="E157" s="5" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="F157" s="9" t="n">
         <v>200</v>
@@ -5914,7 +5914,7 @@
         </is>
       </c>
       <c r="E158" s="5" t="n">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="F158" s="9" t="n">
         <v>200</v>
@@ -5947,7 +5947,7 @@
         </is>
       </c>
       <c r="E159" s="5" t="n">
-        <v>10</v>
+        <v>83</v>
       </c>
       <c r="F159" s="9" t="n">
         <v>200</v>
@@ -5980,7 +5980,7 @@
         </is>
       </c>
       <c r="E160" s="5" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F160" s="9" t="n">
         <v>200</v>
@@ -6013,7 +6013,7 @@
         </is>
       </c>
       <c r="E161" s="5" t="n">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="F161" s="9" t="n">
         <v>200</v>
@@ -6046,7 +6046,7 @@
         </is>
       </c>
       <c r="E162" s="5" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="F162" s="9" t="n">
         <v>200</v>
@@ -6079,7 +6079,7 @@
         </is>
       </c>
       <c r="E163" s="5" t="n">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="F163" s="9" t="n">
         <v>200</v>
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="E164" s="5" t="n">
-        <v>33</v>
+        <v>95</v>
       </c>
       <c r="F164" s="9" t="n">
         <v>200</v>
@@ -6145,7 +6145,7 @@
         </is>
       </c>
       <c r="E165" s="5" t="n">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="F165" s="9" t="n">
         <v>200</v>
@@ -6178,7 +6178,7 @@
         </is>
       </c>
       <c r="E166" s="5" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="F166" s="9" t="n">
         <v>200</v>
@@ -6211,7 +6211,7 @@
         </is>
       </c>
       <c r="E167" s="5" t="n">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="F167" s="9" t="n">
         <v>200</v>
@@ -6244,7 +6244,7 @@
         </is>
       </c>
       <c r="E168" s="5" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F168" s="9" t="n">
         <v>200</v>
@@ -6277,7 +6277,7 @@
         </is>
       </c>
       <c r="E169" s="5" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F169" s="9" t="n">
         <v>200</v>
@@ -6310,7 +6310,7 @@
         </is>
       </c>
       <c r="E170" s="5" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F170" s="9" t="n">
         <v>200</v>
@@ -6343,7 +6343,7 @@
         </is>
       </c>
       <c r="E171" s="5" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F171" s="9" t="n">
         <v>200</v>
@@ -6376,7 +6376,7 @@
         </is>
       </c>
       <c r="E172" s="5" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="F172" s="9" t="n">
         <v>200</v>
@@ -6409,7 +6409,7 @@
         </is>
       </c>
       <c r="E173" s="5" t="n">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="F173" s="9" t="n">
         <v>200</v>
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="E174" s="5" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F174" s="9" t="n">
         <v>200</v>
@@ -6475,7 +6475,7 @@
         </is>
       </c>
       <c r="E175" s="5" t="n">
-        <v>24</v>
+        <v>70</v>
       </c>
       <c r="F175" s="9" t="n">
         <v>200</v>
@@ -6508,7 +6508,7 @@
         </is>
       </c>
       <c r="E176" s="5" t="n">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="F176" s="9" t="n">
         <v>200</v>
@@ -6541,7 +6541,7 @@
         </is>
       </c>
       <c r="E177" s="5" t="n">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="F177" s="9" t="n">
         <v>200</v>
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="E178" s="5" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="F178" s="9" t="n">
         <v>200</v>
@@ -6607,7 +6607,7 @@
         </is>
       </c>
       <c r="E179" s="5" t="n">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="F179" s="9" t="n">
         <v>200</v>
@@ -6640,7 +6640,7 @@
         </is>
       </c>
       <c r="E180" s="5" t="n">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="F180" s="9" t="n">
         <v>200</v>
@@ -6673,7 +6673,7 @@
         </is>
       </c>
       <c r="E181" s="5" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="F181" s="9" t="n">
         <v>200</v>
@@ -6706,7 +6706,7 @@
         </is>
       </c>
       <c r="E182" s="5" t="n">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="F182" s="9" t="n">
         <v>200</v>
@@ -6739,7 +6739,7 @@
         </is>
       </c>
       <c r="E183" s="5" t="n">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="F183" s="9" t="n">
         <v>200</v>
@@ -6772,7 +6772,7 @@
         </is>
       </c>
       <c r="E184" s="5" t="n">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="F184" s="9" t="n">
         <v>200</v>
@@ -6805,7 +6805,7 @@
         </is>
       </c>
       <c r="E185" s="5" t="n">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="F185" s="9" t="n">
         <v>200</v>
@@ -6838,7 +6838,7 @@
         </is>
       </c>
       <c r="E186" s="5" t="n">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="F186" s="9" t="n">
         <v>200</v>
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="E187" s="5" t="n">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="F187" s="9" t="n">
         <v>200</v>
@@ -6904,7 +6904,7 @@
         </is>
       </c>
       <c r="E188" s="5" t="n">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="F188" s="9" t="n">
         <v>200</v>
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="E189" s="5" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F189" s="9" t="n">
         <v>200</v>
@@ -6970,7 +6970,7 @@
         </is>
       </c>
       <c r="E190" s="5" t="n">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="F190" s="9" t="n">
         <v>200</v>
@@ -7003,7 +7003,7 @@
         </is>
       </c>
       <c r="E191" s="5" t="n">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="F191" s="9" t="n">
         <v>200</v>
@@ -7036,7 +7036,7 @@
         </is>
       </c>
       <c r="E192" s="5" t="n">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="F192" s="9" t="n">
         <v>200</v>
@@ -7069,7 +7069,7 @@
         </is>
       </c>
       <c r="E193" s="5" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="F193" s="9" t="n">
         <v>200</v>
@@ -7102,7 +7102,7 @@
         </is>
       </c>
       <c r="E194" s="5" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F194" s="9" t="n">
         <v>200</v>
@@ -7135,7 +7135,7 @@
         </is>
       </c>
       <c r="E195" s="5" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F195" s="9" t="n">
         <v>200</v>
@@ -7168,7 +7168,7 @@
         </is>
       </c>
       <c r="E196" s="5" t="n">
-        <v>78</v>
+        <v>12</v>
       </c>
       <c r="F196" s="9" t="n">
         <v>200</v>
@@ -7201,7 +7201,7 @@
         </is>
       </c>
       <c r="E197" s="5" t="n">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="F197" s="9" t="n">
         <v>200</v>
@@ -7234,7 +7234,7 @@
         </is>
       </c>
       <c r="E198" s="5" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="F198" s="9" t="n">
         <v>200</v>
@@ -7267,7 +7267,7 @@
         </is>
       </c>
       <c r="E199" s="5" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="F199" s="9" t="n">
         <v>200</v>
@@ -7300,7 +7300,7 @@
         </is>
       </c>
       <c r="E200" s="5" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F200" s="9" t="n">
         <v>200</v>
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="E201" s="5" t="n">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="F201" s="9" t="n">
         <v>200</v>
@@ -7366,7 +7366,7 @@
         </is>
       </c>
       <c r="E202" s="5" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="F202" s="9" t="n">
         <v>200</v>
@@ -7399,7 +7399,7 @@
         </is>
       </c>
       <c r="E203" s="5" t="n">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="F203" s="9" t="n">
         <v>200</v>
@@ -7465,7 +7465,7 @@
         </is>
       </c>
       <c r="E205" s="5" t="n">
-        <v>91</v>
+        <v>53</v>
       </c>
       <c r="F205" s="9" t="n">
         <v>200</v>
@@ -7498,7 +7498,7 @@
         </is>
       </c>
       <c r="E206" s="5" t="n">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="F206" s="9" t="n">
         <v>200</v>
@@ -7531,7 +7531,7 @@
         </is>
       </c>
       <c r="E207" s="5" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F207" s="9" t="n">
         <v>200</v>
@@ -7564,7 +7564,7 @@
         </is>
       </c>
       <c r="E208" s="5" t="n">
-        <v>80</v>
+        <v>42</v>
       </c>
       <c r="F208" s="9" t="n">
         <v>200</v>
@@ -7597,7 +7597,7 @@
         </is>
       </c>
       <c r="E209" s="5" t="n">
-        <v>36</v>
+        <v>95</v>
       </c>
       <c r="F209" s="9" t="n">
         <v>200</v>
@@ -7630,7 +7630,7 @@
         </is>
       </c>
       <c r="E210" s="5" t="n">
-        <v>94</v>
+        <v>23</v>
       </c>
       <c r="F210" s="9" t="n">
         <v>200</v>
@@ -7663,7 +7663,7 @@
         </is>
       </c>
       <c r="E211" s="5" t="n">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="F211" s="9" t="n">
         <v>200</v>
@@ -7696,7 +7696,7 @@
         </is>
       </c>
       <c r="E212" s="5" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F212" s="9" t="n">
         <v>200</v>
@@ -7729,7 +7729,7 @@
         </is>
       </c>
       <c r="E213" s="5" t="n">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="F213" s="9" t="n">
         <v>200</v>
@@ -7762,7 +7762,7 @@
         </is>
       </c>
       <c r="E214" s="5" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="F214" s="9" t="n">
         <v>200</v>
@@ -7795,7 +7795,7 @@
         </is>
       </c>
       <c r="E215" s="5" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F215" s="9" t="n">
         <v>200</v>
@@ -7828,7 +7828,7 @@
         </is>
       </c>
       <c r="E216" s="5" t="n">
-        <v>82</v>
+        <v>31</v>
       </c>
       <c r="F216" s="9" t="n">
         <v>200</v>
@@ -7861,7 +7861,7 @@
         </is>
       </c>
       <c r="E217" s="5" t="n">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="F217" s="9" t="n">
         <v>200</v>
@@ -7894,7 +7894,7 @@
         </is>
       </c>
       <c r="E218" s="5" t="n">
-        <v>86</v>
+        <v>23</v>
       </c>
       <c r="F218" s="9" t="n">
         <v>200</v>
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="E219" s="5" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F219" s="9" t="n">
         <v>200</v>
@@ -7960,7 +7960,7 @@
         </is>
       </c>
       <c r="E220" s="5" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="F220" s="9" t="n">
         <v>200</v>
@@ -7993,7 +7993,7 @@
         </is>
       </c>
       <c r="E221" s="5" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F221" s="9" t="n">
         <v>200</v>
@@ -8026,7 +8026,7 @@
         </is>
       </c>
       <c r="E222" s="5" t="n">
-        <v>49</v>
+        <v>89</v>
       </c>
       <c r="F222" s="9" t="n">
         <v>200</v>
@@ -8059,7 +8059,7 @@
         </is>
       </c>
       <c r="E223" s="5" t="n">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="F223" s="9" t="n">
         <v>200</v>
@@ -8092,7 +8092,7 @@
         </is>
       </c>
       <c r="E224" s="5" t="n">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="F224" s="9" t="n">
         <v>200</v>
@@ -8125,7 +8125,7 @@
         </is>
       </c>
       <c r="E225" s="5" t="n">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="F225" s="9" t="n">
         <v>200</v>
@@ -8158,7 +8158,7 @@
         </is>
       </c>
       <c r="E226" s="5" t="n">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="F226" s="9" t="n">
         <v>200</v>
@@ -8191,7 +8191,7 @@
         </is>
       </c>
       <c r="E227" s="5" t="n">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="F227" s="9" t="n">
         <v>200</v>
@@ -8224,7 +8224,7 @@
         </is>
       </c>
       <c r="E228" s="5" t="n">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="F228" s="9" t="n">
         <v>200</v>
@@ -8257,7 +8257,7 @@
         </is>
       </c>
       <c r="E229" s="5" t="n">
-        <v>15</v>
+        <v>64</v>
       </c>
       <c r="F229" s="9" t="n">
         <v>200</v>
@@ -8290,7 +8290,7 @@
         </is>
       </c>
       <c r="E230" s="5" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="F230" s="9" t="n">
         <v>200</v>
@@ -8323,7 +8323,7 @@
         </is>
       </c>
       <c r="E231" s="5" t="n">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="F231" s="9" t="n">
         <v>200</v>
@@ -8356,7 +8356,7 @@
         </is>
       </c>
       <c r="E232" s="5" t="n">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="F232" s="9" t="n">
         <v>200</v>
@@ -8389,7 +8389,7 @@
         </is>
       </c>
       <c r="E233" s="5" t="n">
-        <v>14</v>
+        <v>76</v>
       </c>
       <c r="F233" s="9" t="n">
         <v>200</v>
@@ -8422,7 +8422,7 @@
         </is>
       </c>
       <c r="E234" s="5" t="n">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="F234" s="9" t="n">
         <v>200</v>
@@ -8455,7 +8455,7 @@
         </is>
       </c>
       <c r="E235" s="5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F235" s="9" t="n">
         <v>200</v>
@@ -8488,7 +8488,7 @@
         </is>
       </c>
       <c r="E236" s="5" t="n">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="F236" s="9" t="n">
         <v>200</v>
@@ -8521,7 +8521,7 @@
         </is>
       </c>
       <c r="E237" s="5" t="n">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="F237" s="9" t="n">
         <v>200</v>
@@ -8554,7 +8554,7 @@
         </is>
       </c>
       <c r="E238" s="5" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F238" s="9" t="n">
         <v>200</v>
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="E239" s="5" t="n">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="F239" s="9" t="n">
         <v>200</v>
@@ -8620,7 +8620,7 @@
         </is>
       </c>
       <c r="E240" s="5" t="n">
-        <v>72</v>
+        <v>13</v>
       </c>
       <c r="F240" s="9" t="n">
         <v>200</v>
@@ -8653,7 +8653,7 @@
         </is>
       </c>
       <c r="E241" s="5" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F241" s="9" t="n">
         <v>200</v>
@@ -8686,7 +8686,7 @@
         </is>
       </c>
       <c r="E242" s="5" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F242" s="9" t="n">
         <v>200</v>
@@ -8719,7 +8719,7 @@
         </is>
       </c>
       <c r="E243" s="5" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="F243" s="9" t="n">
         <v>200</v>
@@ -8752,7 +8752,7 @@
         </is>
       </c>
       <c r="E244" s="5" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F244" s="9" t="n">
         <v>200</v>
@@ -8785,7 +8785,7 @@
         </is>
       </c>
       <c r="E245" s="5" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="F245" s="9" t="n">
         <v>200</v>
@@ -8818,7 +8818,7 @@
         </is>
       </c>
       <c r="E246" s="5" t="n">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="F246" s="9" t="n">
         <v>200</v>
@@ -8851,7 +8851,7 @@
         </is>
       </c>
       <c r="E247" s="5" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="F247" s="9" t="n">
         <v>200</v>
@@ -8884,7 +8884,7 @@
         </is>
       </c>
       <c r="E248" s="5" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F248" s="9" t="n">
         <v>200</v>
@@ -8917,7 +8917,7 @@
         </is>
       </c>
       <c r="E249" s="5" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="F249" s="9" t="n">
         <v>200</v>
@@ -8950,7 +8950,7 @@
         </is>
       </c>
       <c r="E250" s="5" t="n">
-        <v>30</v>
+        <v>91</v>
       </c>
       <c r="F250" s="9" t="n">
         <v>200</v>
@@ -8983,7 +8983,7 @@
         </is>
       </c>
       <c r="E251" s="5" t="n">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="F251" s="9" t="n">
         <v>200</v>
@@ -9016,7 +9016,7 @@
         </is>
       </c>
       <c r="E252" s="5" t="n">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="F252" s="9" t="n">
         <v>200</v>
@@ -9049,7 +9049,7 @@
         </is>
       </c>
       <c r="E253" s="5" t="n">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="F253" s="9" t="n">
         <v>200</v>
@@ -9082,7 +9082,7 @@
         </is>
       </c>
       <c r="E254" s="5" t="n">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="F254" s="9" t="n">
         <v>200</v>
@@ -9115,7 +9115,7 @@
         </is>
       </c>
       <c r="E255" s="5" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F255" s="9" t="n">
         <v>200</v>
@@ -9148,7 +9148,7 @@
         </is>
       </c>
       <c r="E256" s="5" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="F256" s="9" t="n">
         <v>200</v>
@@ -9181,7 +9181,7 @@
         </is>
       </c>
       <c r="E257" s="5" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="F257" s="9" t="n">
         <v>200</v>
@@ -9214,7 +9214,7 @@
         </is>
       </c>
       <c r="E258" s="5" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="F258" s="9" t="n">
         <v>200</v>
@@ -9247,7 +9247,7 @@
         </is>
       </c>
       <c r="E259" s="5" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F259" s="9" t="n">
         <v>200</v>
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="E260" s="5" t="n">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="F260" s="9" t="n">
         <v>200</v>
@@ -9313,7 +9313,7 @@
         </is>
       </c>
       <c r="E261" s="5" t="n">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="F261" s="9" t="n">
         <v>200</v>
@@ -9346,7 +9346,7 @@
         </is>
       </c>
       <c r="E262" s="5" t="n">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="F262" s="9" t="n">
         <v>200</v>
@@ -9379,7 +9379,7 @@
         </is>
       </c>
       <c r="E263" s="5" t="n">
-        <v>39</v>
+        <v>83</v>
       </c>
       <c r="F263" s="9" t="n">
         <v>200</v>
@@ -9412,7 +9412,7 @@
         </is>
       </c>
       <c r="E264" s="5" t="n">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="F264" s="9" t="n">
         <v>200</v>
@@ -9445,7 +9445,7 @@
         </is>
       </c>
       <c r="E265" s="5" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F265" s="9" t="n">
         <v>200</v>
@@ -9478,7 +9478,7 @@
         </is>
       </c>
       <c r="E266" s="5" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="F266" s="9" t="n">
         <v>200</v>
@@ -9511,7 +9511,7 @@
         </is>
       </c>
       <c r="E267" s="5" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F267" s="9" t="n">
         <v>200</v>
@@ -9544,7 +9544,7 @@
         </is>
       </c>
       <c r="E268" s="5" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F268" s="9" t="n">
         <v>200</v>
@@ -9610,7 +9610,7 @@
         </is>
       </c>
       <c r="E270" s="5" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="F270" s="9" t="n">
         <v>200</v>
@@ -9643,7 +9643,7 @@
         </is>
       </c>
       <c r="E271" s="5" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F271" s="9" t="n">
         <v>200</v>
@@ -9676,7 +9676,7 @@
         </is>
       </c>
       <c r="E272" s="5" t="n">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="F272" s="9" t="n">
         <v>200</v>
@@ -9709,7 +9709,7 @@
         </is>
       </c>
       <c r="E273" s="5" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F273" s="9" t="n">
         <v>200</v>
@@ -9742,7 +9742,7 @@
         </is>
       </c>
       <c r="E274" s="5" t="n">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="F274" s="9" t="n">
         <v>200</v>
@@ -9775,7 +9775,7 @@
         </is>
       </c>
       <c r="E275" s="5" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F275" s="9" t="n">
         <v>200</v>
@@ -9808,7 +9808,7 @@
         </is>
       </c>
       <c r="E276" s="5" t="n">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="F276" s="9" t="n">
         <v>200</v>
@@ -9841,7 +9841,7 @@
         </is>
       </c>
       <c r="E277" s="5" t="n">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="F277" s="9" t="n">
         <v>200</v>
@@ -9874,7 +9874,7 @@
         </is>
       </c>
       <c r="E278" s="5" t="n">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="F278" s="9" t="n">
         <v>200</v>
@@ -9907,7 +9907,7 @@
         </is>
       </c>
       <c r="E279" s="5" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="F279" s="9" t="n">
         <v>200</v>
@@ -9940,7 +9940,7 @@
         </is>
       </c>
       <c r="E280" s="5" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="F280" s="9" t="n">
         <v>200</v>
@@ -9973,7 +9973,7 @@
         </is>
       </c>
       <c r="E281" s="5" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F281" s="9" t="n">
         <v>200</v>
@@ -10006,7 +10006,7 @@
         </is>
       </c>
       <c r="E282" s="5" t="n">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="F282" s="9" t="n">
         <v>200</v>
@@ -10039,7 +10039,7 @@
         </is>
       </c>
       <c r="E283" s="5" t="n">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="F283" s="9" t="n">
         <v>200</v>
@@ -10072,7 +10072,7 @@
         </is>
       </c>
       <c r="E284" s="5" t="n">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="F284" s="9" t="n">
         <v>200</v>
@@ -10105,7 +10105,7 @@
         </is>
       </c>
       <c r="E285" s="5" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F285" s="9" t="n">
         <v>200</v>
@@ -10138,7 +10138,7 @@
         </is>
       </c>
       <c r="E286" s="5" t="n">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="F286" s="9" t="n">
         <v>200</v>
@@ -10171,7 +10171,7 @@
         </is>
       </c>
       <c r="E287" s="5" t="n">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="F287" s="9" t="n">
         <v>200</v>
@@ -10204,7 +10204,7 @@
         </is>
       </c>
       <c r="E288" s="5" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="F288" s="9" t="n">
         <v>200</v>
@@ -10237,7 +10237,7 @@
         </is>
       </c>
       <c r="E289" s="5" t="n">
-        <v>41</v>
+        <v>87</v>
       </c>
       <c r="F289" s="9" t="n">
         <v>200</v>
@@ -10270,7 +10270,7 @@
         </is>
       </c>
       <c r="E290" s="5" t="n">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="F290" s="9" t="n">
         <v>200</v>
@@ -10303,7 +10303,7 @@
         </is>
       </c>
       <c r="E291" s="5" t="n">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="F291" s="9" t="n">
         <v>200</v>
@@ -10336,7 +10336,7 @@
         </is>
       </c>
       <c r="E292" s="5" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="F292" s="9" t="n">
         <v>200</v>
@@ -10369,7 +10369,7 @@
         </is>
       </c>
       <c r="E293" s="5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F293" s="9" t="n">
         <v>200</v>
@@ -10402,7 +10402,7 @@
         </is>
       </c>
       <c r="E294" s="5" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="F294" s="9" t="n">
         <v>200</v>
@@ -10435,7 +10435,7 @@
         </is>
       </c>
       <c r="E295" s="5" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="F295" s="9" t="n">
         <v>200</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="E296" s="5" t="n">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="F296" s="9" t="n">
         <v>200</v>
@@ -10501,7 +10501,7 @@
         </is>
       </c>
       <c r="E297" s="5" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="F297" s="9" t="n">
         <v>200</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="E298" s="5" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F298" s="9" t="n">
         <v>200</v>
@@ -10567,7 +10567,7 @@
         </is>
       </c>
       <c r="E299" s="5" t="n">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="F299" s="9" t="n">
         <v>200</v>
@@ -10600,7 +10600,7 @@
         </is>
       </c>
       <c r="E300" s="5" t="n">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="F300" s="9" t="n">
         <v>200</v>
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="E301" s="5" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F301" s="9" t="n">
         <v>200</v>

</xml_diff>

<commit_message>
Include Appium and Selenium Excel report in E2E artifact upload
</commit_message>
<xml_diff>
--- a/k6_load_test_report.xlsx
+++ b/k6_load_test_report.xlsx
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="F2" s="9" t="n">
         <v>200</v>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>200</v>
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>200</v>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>200</v>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>200</v>
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>200</v>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>200</v>
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>200</v>
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>200</v>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>22</v>
+        <v>66</v>
       </c>
       <c r="F11" s="9" t="n">
         <v>200</v>
@@ -1096,7 +1096,7 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="F12" s="9" t="n">
         <v>200</v>
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F13" s="9" t="n">
         <v>200</v>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F14" s="9" t="n">
         <v>200</v>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F15" s="9" t="n">
         <v>200</v>
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F16" s="9" t="n">
         <v>200</v>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F17" s="9" t="n">
         <v>200</v>
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F18" s="9" t="n">
         <v>200</v>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="F19" s="9" t="n">
         <v>200</v>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>46</v>
+        <v>89</v>
       </c>
       <c r="F20" s="9" t="n">
         <v>200</v>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>88</v>
+        <v>26</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>200</v>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="F22" s="9" t="n">
         <v>200</v>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F23" s="9" t="n">
         <v>200</v>
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="F24" s="9" t="n">
         <v>200</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="F25" s="9" t="n">
         <v>200</v>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>200</v>
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="F27" s="9" t="n">
         <v>200</v>
@@ -1624,7 +1624,7 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="F28" s="9" t="n">
         <v>200</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="F29" s="9" t="n">
         <v>200</v>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>200</v>
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="F31" s="9" t="n">
         <v>200</v>
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="F32" s="9" t="n">
         <v>200</v>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="F33" s="9" t="n">
         <v>200</v>
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="F34" s="9" t="n">
         <v>200</v>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="F35" s="9" t="n">
         <v>200</v>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F36" s="9" t="n">
         <v>200</v>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>200</v>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>200</v>
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F39" s="9" t="n">
         <v>200</v>
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="E40" s="5" t="n">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="F40" s="9" t="n">
         <v>200</v>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="F41" s="9" t="n">
         <v>200</v>
@@ -2086,7 +2086,7 @@
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F42" s="9" t="n">
         <v>200</v>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="E43" s="5" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F43" s="9" t="n">
         <v>200</v>
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>200</v>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F45" s="9" t="n">
         <v>200</v>
@@ -2218,7 +2218,7 @@
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="F46" s="9" t="n">
         <v>200</v>
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>37</v>
+        <v>95</v>
       </c>
       <c r="F47" s="9" t="n">
         <v>200</v>
@@ -2284,7 +2284,7 @@
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="F48" s="9" t="n">
         <v>200</v>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="F49" s="9" t="n">
         <v>200</v>
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="F50" s="9" t="n">
         <v>200</v>
@@ -2383,7 +2383,7 @@
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>87</v>
+        <v>22</v>
       </c>
       <c r="F51" s="9" t="n">
         <v>200</v>
@@ -2416,7 +2416,7 @@
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="F52" s="9" t="n">
         <v>200</v>
@@ -2449,7 +2449,7 @@
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="F53" s="9" t="n">
         <v>200</v>
@@ -2482,7 +2482,7 @@
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F54" s="9" t="n">
         <v>200</v>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="F55" s="9" t="n">
         <v>200</v>
@@ -2548,7 +2548,7 @@
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>79</v>
+        <v>57</v>
       </c>
       <c r="F56" s="9" t="n">
         <v>200</v>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="F57" s="9" t="n">
         <v>200</v>
@@ -2614,7 +2614,7 @@
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="F58" s="9" t="n">
         <v>200</v>
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="F59" s="9" t="n">
         <v>200</v>
@@ -2680,7 +2680,7 @@
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>11</v>
+        <v>71</v>
       </c>
       <c r="F60" s="9" t="n">
         <v>200</v>
@@ -2713,7 +2713,7 @@
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="F61" s="9" t="n">
         <v>200</v>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="F62" s="9" t="n">
         <v>200</v>
@@ -2779,7 +2779,7 @@
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="F63" s="9" t="n">
         <v>200</v>
@@ -2812,7 +2812,7 @@
         </is>
       </c>
       <c r="E64" s="5" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F64" s="9" t="n">
         <v>200</v>
@@ -2845,7 +2845,7 @@
         </is>
       </c>
       <c r="E65" s="5" t="n">
-        <v>95</v>
+        <v>42</v>
       </c>
       <c r="F65" s="9" t="n">
         <v>200</v>
@@ -2878,7 +2878,7 @@
         </is>
       </c>
       <c r="E66" s="5" t="n">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="F66" s="9" t="n">
         <v>200</v>
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="E67" s="5" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="F67" s="9" t="n">
         <v>200</v>
@@ -2944,7 +2944,7 @@
         </is>
       </c>
       <c r="E68" s="5" t="n">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="F68" s="9" t="n">
         <v>200</v>
@@ -2977,7 +2977,7 @@
         </is>
       </c>
       <c r="E69" s="5" t="n">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="F69" s="9" t="n">
         <v>200</v>
@@ -3010,7 +3010,7 @@
         </is>
       </c>
       <c r="E70" s="5" t="n">
-        <v>27</v>
+        <v>78</v>
       </c>
       <c r="F70" s="9" t="n">
         <v>200</v>
@@ -3043,7 +3043,7 @@
         </is>
       </c>
       <c r="E71" s="5" t="n">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="F71" s="9" t="n">
         <v>200</v>
@@ -3076,7 +3076,7 @@
         </is>
       </c>
       <c r="E72" s="5" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>200</v>
@@ -3109,7 +3109,7 @@
         </is>
       </c>
       <c r="E73" s="5" t="n">
-        <v>94</v>
+        <v>41</v>
       </c>
       <c r="F73" s="9" t="n">
         <v>200</v>
@@ -3142,7 +3142,7 @@
         </is>
       </c>
       <c r="E74" s="5" t="n">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="F74" s="9" t="n">
         <v>200</v>
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="E75" s="5" t="n">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="F75" s="9" t="n">
         <v>200</v>
@@ -3208,7 +3208,7 @@
         </is>
       </c>
       <c r="E76" s="5" t="n">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="F76" s="9" t="n">
         <v>200</v>
@@ -3241,7 +3241,7 @@
         </is>
       </c>
       <c r="E77" s="5" t="n">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="F77" s="9" t="n">
         <v>200</v>
@@ -3274,7 +3274,7 @@
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F78" s="9" t="n">
         <v>200</v>
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="E79" s="5" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="F79" s="9" t="n">
         <v>200</v>
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="E80" s="5" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F80" s="9" t="n">
         <v>200</v>
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="E81" s="5" t="n">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="F81" s="9" t="n">
         <v>200</v>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="E82" s="5" t="n">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="F82" s="9" t="n">
         <v>200</v>
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="E83" s="5" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="F83" s="9" t="n">
         <v>200</v>
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="E85" s="5" t="n">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="F85" s="9" t="n">
         <v>200</v>
@@ -3538,7 +3538,7 @@
         </is>
       </c>
       <c r="E86" s="5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F86" s="9" t="n">
         <v>200</v>
@@ -3571,7 +3571,7 @@
         </is>
       </c>
       <c r="E87" s="5" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="F87" s="9" t="n">
         <v>200</v>
@@ -3604,7 +3604,7 @@
         </is>
       </c>
       <c r="E88" s="5" t="n">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="F88" s="9" t="n">
         <v>200</v>
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="E89" s="5" t="n">
-        <v>33</v>
+        <v>89</v>
       </c>
       <c r="F89" s="9" t="n">
         <v>200</v>
@@ -3670,7 +3670,7 @@
         </is>
       </c>
       <c r="E90" s="5" t="n">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="F90" s="9" t="n">
         <v>200</v>
@@ -3703,7 +3703,7 @@
         </is>
       </c>
       <c r="E91" s="5" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="F91" s="9" t="n">
         <v>200</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="E92" s="5" t="n">
-        <v>88</v>
+        <v>16</v>
       </c>
       <c r="F92" s="9" t="n">
         <v>200</v>
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="E93" s="5" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="F93" s="9" t="n">
         <v>200</v>
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="E94" s="5" t="n">
-        <v>55</v>
+        <v>87</v>
       </c>
       <c r="F94" s="9" t="n">
         <v>200</v>
@@ -3835,7 +3835,7 @@
         </is>
       </c>
       <c r="E95" s="5" t="n">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="F95" s="9" t="n">
         <v>200</v>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="E96" s="5" t="n">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="F96" s="9" t="n">
         <v>200</v>
@@ -3901,7 +3901,7 @@
         </is>
       </c>
       <c r="E97" s="5" t="n">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="F97" s="9" t="n">
         <v>200</v>
@@ -3934,7 +3934,7 @@
         </is>
       </c>
       <c r="E98" s="5" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F98" s="9" t="n">
         <v>200</v>
@@ -3967,7 +3967,7 @@
         </is>
       </c>
       <c r="E99" s="5" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F99" s="9" t="n">
         <v>200</v>
@@ -4000,7 +4000,7 @@
         </is>
       </c>
       <c r="E100" s="5" t="n">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="F100" s="9" t="n">
         <v>200</v>
@@ -4033,7 +4033,7 @@
         </is>
       </c>
       <c r="E101" s="5" t="n">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F101" s="9" t="n">
         <v>200</v>
@@ -4066,7 +4066,7 @@
         </is>
       </c>
       <c r="E102" s="5" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="F102" s="9" t="n">
         <v>200</v>
@@ -4099,7 +4099,7 @@
         </is>
       </c>
       <c r="E103" s="5" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F103" s="9" t="n">
         <v>200</v>
@@ -4132,7 +4132,7 @@
         </is>
       </c>
       <c r="E104" s="5" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="F104" s="9" t="n">
         <v>200</v>
@@ -4165,7 +4165,7 @@
         </is>
       </c>
       <c r="E105" s="5" t="n">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="F105" s="9" t="n">
         <v>200</v>
@@ -4198,7 +4198,7 @@
         </is>
       </c>
       <c r="E106" s="5" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="F106" s="9" t="n">
         <v>200</v>
@@ -4231,7 +4231,7 @@
         </is>
       </c>
       <c r="E107" s="5" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F107" s="9" t="n">
         <v>200</v>
@@ -4264,7 +4264,7 @@
         </is>
       </c>
       <c r="E108" s="5" t="n">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="F108" s="9" t="n">
         <v>200</v>
@@ -4297,7 +4297,7 @@
         </is>
       </c>
       <c r="E109" s="5" t="n">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="F109" s="9" t="n">
         <v>200</v>
@@ -4330,7 +4330,7 @@
         </is>
       </c>
       <c r="E110" s="5" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="F110" s="9" t="n">
         <v>200</v>
@@ -4363,7 +4363,7 @@
         </is>
       </c>
       <c r="E111" s="5" t="n">
-        <v>14</v>
+        <v>93</v>
       </c>
       <c r="F111" s="9" t="n">
         <v>200</v>
@@ -4396,7 +4396,7 @@
         </is>
       </c>
       <c r="E112" s="5" t="n">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="F112" s="9" t="n">
         <v>200</v>
@@ -4429,7 +4429,7 @@
         </is>
       </c>
       <c r="E113" s="5" t="n">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="F113" s="9" t="n">
         <v>200</v>
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="E114" s="5" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F114" s="9" t="n">
         <v>200</v>
@@ -4495,7 +4495,7 @@
         </is>
       </c>
       <c r="E115" s="5" t="n">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="F115" s="9" t="n">
         <v>200</v>
@@ -4528,7 +4528,7 @@
         </is>
       </c>
       <c r="E116" s="5" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="F116" s="9" t="n">
         <v>200</v>
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="E117" s="5" t="n">
-        <v>35</v>
+        <v>94</v>
       </c>
       <c r="F117" s="9" t="n">
         <v>200</v>
@@ -4594,7 +4594,7 @@
         </is>
       </c>
       <c r="E118" s="5" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="F118" s="9" t="n">
         <v>200</v>
@@ -4627,7 +4627,7 @@
         </is>
       </c>
       <c r="E119" s="5" t="n">
-        <v>51</v>
+        <v>88</v>
       </c>
       <c r="F119" s="9" t="n">
         <v>200</v>
@@ -4660,7 +4660,7 @@
         </is>
       </c>
       <c r="E120" s="5" t="n">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="F120" s="9" t="n">
         <v>200</v>
@@ -4693,7 +4693,7 @@
         </is>
       </c>
       <c r="E121" s="5" t="n">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="F121" s="9" t="n">
         <v>200</v>
@@ -4726,7 +4726,7 @@
         </is>
       </c>
       <c r="E122" s="5" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F122" s="9" t="n">
         <v>200</v>
@@ -4759,7 +4759,7 @@
         </is>
       </c>
       <c r="E123" s="5" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F123" s="9" t="n">
         <v>200</v>
@@ -4792,7 +4792,7 @@
         </is>
       </c>
       <c r="E124" s="5" t="n">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="F124" s="9" t="n">
         <v>200</v>
@@ -4825,7 +4825,7 @@
         </is>
       </c>
       <c r="E125" s="5" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="F125" s="9" t="n">
         <v>200</v>
@@ -4858,7 +4858,7 @@
         </is>
       </c>
       <c r="E126" s="5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F126" s="9" t="n">
         <v>200</v>
@@ -4891,7 +4891,7 @@
         </is>
       </c>
       <c r="E127" s="5" t="n">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="F127" s="9" t="n">
         <v>200</v>
@@ -4924,7 +4924,7 @@
         </is>
       </c>
       <c r="E128" s="5" t="n">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="F128" s="9" t="n">
         <v>200</v>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="E129" s="5" t="n">
-        <v>62</v>
+        <v>24</v>
       </c>
       <c r="F129" s="9" t="n">
         <v>200</v>
@@ -4990,7 +4990,7 @@
         </is>
       </c>
       <c r="E130" s="5" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="F130" s="9" t="n">
         <v>200</v>
@@ -5023,7 +5023,7 @@
         </is>
       </c>
       <c r="E131" s="5" t="n">
-        <v>85</v>
+        <v>48</v>
       </c>
       <c r="F131" s="9" t="n">
         <v>200</v>
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="E132" s="5" t="n">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="F132" s="9" t="n">
         <v>200</v>
@@ -5089,7 +5089,7 @@
         </is>
       </c>
       <c r="E133" s="5" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="F133" s="9" t="n">
         <v>200</v>
@@ -5122,7 +5122,7 @@
         </is>
       </c>
       <c r="E134" s="5" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F134" s="9" t="n">
         <v>200</v>
@@ -5155,7 +5155,7 @@
         </is>
       </c>
       <c r="E135" s="5" t="n">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="F135" s="9" t="n">
         <v>200</v>
@@ -5188,7 +5188,7 @@
         </is>
       </c>
       <c r="E136" s="5" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F136" s="9" t="n">
         <v>200</v>
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="E137" s="5" t="n">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="F137" s="9" t="n">
         <v>200</v>
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="E138" s="5" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F138" s="9" t="n">
         <v>200</v>
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="E139" s="5" t="n">
-        <v>94</v>
+        <v>26</v>
       </c>
       <c r="F139" s="9" t="n">
         <v>200</v>
@@ -5320,7 +5320,7 @@
         </is>
       </c>
       <c r="E140" s="5" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="F140" s="9" t="n">
         <v>200</v>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="E141" s="5" t="n">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="F141" s="9" t="n">
         <v>200</v>
@@ -5386,7 +5386,7 @@
         </is>
       </c>
       <c r="E142" s="5" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F142" s="9" t="n">
         <v>200</v>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="E143" s="5" t="n">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="F143" s="9" t="n">
         <v>200</v>
@@ -5452,7 +5452,7 @@
         </is>
       </c>
       <c r="E144" s="5" t="n">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="F144" s="9" t="n">
         <v>200</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="E145" s="5" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F145" s="9" t="n">
         <v>200</v>
@@ -5518,7 +5518,7 @@
         </is>
       </c>
       <c r="E146" s="5" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F146" s="9" t="n">
         <v>200</v>
@@ -5551,7 +5551,7 @@
         </is>
       </c>
       <c r="E147" s="5" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="F147" s="9" t="n">
         <v>200</v>
@@ -5584,7 +5584,7 @@
         </is>
       </c>
       <c r="E148" s="5" t="n">
-        <v>33</v>
+        <v>77</v>
       </c>
       <c r="F148" s="9" t="n">
         <v>200</v>
@@ -5617,7 +5617,7 @@
         </is>
       </c>
       <c r="E149" s="5" t="n">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="F149" s="9" t="n">
         <v>200</v>
@@ -5650,7 +5650,7 @@
         </is>
       </c>
       <c r="E150" s="5" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="F150" s="9" t="n">
         <v>200</v>
@@ -5683,7 +5683,7 @@
         </is>
       </c>
       <c r="E151" s="5" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="F151" s="9" t="n">
         <v>200</v>
@@ -5716,7 +5716,7 @@
         </is>
       </c>
       <c r="E152" s="5" t="n">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="F152" s="9" t="n">
         <v>200</v>
@@ -5749,7 +5749,7 @@
         </is>
       </c>
       <c r="E153" s="5" t="n">
-        <v>28</v>
+        <v>84</v>
       </c>
       <c r="F153" s="9" t="n">
         <v>200</v>
@@ -5782,7 +5782,7 @@
         </is>
       </c>
       <c r="E154" s="5" t="n">
-        <v>94</v>
+        <v>45</v>
       </c>
       <c r="F154" s="9" t="n">
         <v>200</v>
@@ -5815,7 +5815,7 @@
         </is>
       </c>
       <c r="E155" s="5" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="F155" s="9" t="n">
         <v>200</v>
@@ -5848,7 +5848,7 @@
         </is>
       </c>
       <c r="E156" s="5" t="n">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="F156" s="9" t="n">
         <v>200</v>
@@ -5881,7 +5881,7 @@
         </is>
       </c>
       <c r="E157" s="5" t="n">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="F157" s="9" t="n">
         <v>200</v>
@@ -5914,7 +5914,7 @@
         </is>
       </c>
       <c r="E158" s="5" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="F158" s="9" t="n">
         <v>200</v>
@@ -5947,7 +5947,7 @@
         </is>
       </c>
       <c r="E159" s="5" t="n">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="F159" s="9" t="n">
         <v>200</v>
@@ -5980,7 +5980,7 @@
         </is>
       </c>
       <c r="E160" s="5" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="F160" s="9" t="n">
         <v>200</v>
@@ -6013,7 +6013,7 @@
         </is>
       </c>
       <c r="E161" s="5" t="n">
-        <v>29</v>
+        <v>95</v>
       </c>
       <c r="F161" s="9" t="n">
         <v>200</v>
@@ -6046,7 +6046,7 @@
         </is>
       </c>
       <c r="E162" s="5" t="n">
-        <v>64</v>
+        <v>19</v>
       </c>
       <c r="F162" s="9" t="n">
         <v>200</v>
@@ -6079,7 +6079,7 @@
         </is>
       </c>
       <c r="E163" s="5" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="F163" s="9" t="n">
         <v>200</v>
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="E164" s="5" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F164" s="9" t="n">
         <v>200</v>
@@ -6145,7 +6145,7 @@
         </is>
       </c>
       <c r="E165" s="5" t="n">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="F165" s="9" t="n">
         <v>200</v>
@@ -6178,7 +6178,7 @@
         </is>
       </c>
       <c r="E166" s="5" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="F166" s="9" t="n">
         <v>200</v>
@@ -6211,7 +6211,7 @@
         </is>
       </c>
       <c r="E167" s="5" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="F167" s="9" t="n">
         <v>200</v>
@@ -6244,7 +6244,7 @@
         </is>
       </c>
       <c r="E168" s="5" t="n">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="F168" s="9" t="n">
         <v>200</v>
@@ -6277,7 +6277,7 @@
         </is>
       </c>
       <c r="E169" s="5" t="n">
-        <v>29</v>
+        <v>87</v>
       </c>
       <c r="F169" s="9" t="n">
         <v>200</v>
@@ -6310,7 +6310,7 @@
         </is>
       </c>
       <c r="E170" s="5" t="n">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="F170" s="9" t="n">
         <v>200</v>
@@ -6343,7 +6343,7 @@
         </is>
       </c>
       <c r="E171" s="5" t="n">
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="F171" s="9" t="n">
         <v>200</v>
@@ -6409,7 +6409,7 @@
         </is>
       </c>
       <c r="E173" s="5" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="F173" s="9" t="n">
         <v>200</v>
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="E174" s="5" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="F174" s="9" t="n">
         <v>200</v>
@@ -6475,7 +6475,7 @@
         </is>
       </c>
       <c r="E175" s="5" t="n">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="F175" s="9" t="n">
         <v>200</v>
@@ -6508,7 +6508,7 @@
         </is>
       </c>
       <c r="E176" s="5" t="n">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="F176" s="9" t="n">
         <v>200</v>
@@ -6541,7 +6541,7 @@
         </is>
       </c>
       <c r="E177" s="5" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F177" s="9" t="n">
         <v>200</v>
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="E178" s="5" t="n">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="F178" s="9" t="n">
         <v>200</v>
@@ -6607,7 +6607,7 @@
         </is>
       </c>
       <c r="E179" s="5" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="F179" s="9" t="n">
         <v>200</v>
@@ -6640,7 +6640,7 @@
         </is>
       </c>
       <c r="E180" s="5" t="n">
-        <v>78</v>
+        <v>12</v>
       </c>
       <c r="F180" s="9" t="n">
         <v>200</v>
@@ -6673,7 +6673,7 @@
         </is>
       </c>
       <c r="E181" s="5" t="n">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="F181" s="9" t="n">
         <v>200</v>
@@ -6706,7 +6706,7 @@
         </is>
       </c>
       <c r="E182" s="5" t="n">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="F182" s="9" t="n">
         <v>200</v>
@@ -6739,7 +6739,7 @@
         </is>
       </c>
       <c r="E183" s="5" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F183" s="9" t="n">
         <v>200</v>
@@ -6772,7 +6772,7 @@
         </is>
       </c>
       <c r="E184" s="5" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="F184" s="9" t="n">
         <v>200</v>
@@ -6805,7 +6805,7 @@
         </is>
       </c>
       <c r="E185" s="5" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="F185" s="9" t="n">
         <v>200</v>
@@ -6838,7 +6838,7 @@
         </is>
       </c>
       <c r="E186" s="5" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="F186" s="9" t="n">
         <v>200</v>
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="E187" s="5" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="F187" s="9" t="n">
         <v>200</v>
@@ -6904,7 +6904,7 @@
         </is>
       </c>
       <c r="E188" s="5" t="n">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="F188" s="9" t="n">
         <v>200</v>
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="E189" s="5" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F189" s="9" t="n">
         <v>200</v>
@@ -6970,7 +6970,7 @@
         </is>
       </c>
       <c r="E190" s="5" t="n">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="F190" s="9" t="n">
         <v>200</v>
@@ -7003,7 +7003,7 @@
         </is>
       </c>
       <c r="E191" s="5" t="n">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="F191" s="9" t="n">
         <v>200</v>
@@ -7036,7 +7036,7 @@
         </is>
       </c>
       <c r="E192" s="5" t="n">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="F192" s="9" t="n">
         <v>200</v>
@@ -7069,7 +7069,7 @@
         </is>
       </c>
       <c r="E193" s="5" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="F193" s="9" t="n">
         <v>200</v>
@@ -7102,7 +7102,7 @@
         </is>
       </c>
       <c r="E194" s="5" t="n">
-        <v>15</v>
+        <v>67</v>
       </c>
       <c r="F194" s="9" t="n">
         <v>200</v>
@@ -7135,7 +7135,7 @@
         </is>
       </c>
       <c r="E195" s="5" t="n">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F195" s="9" t="n">
         <v>200</v>
@@ -7168,7 +7168,7 @@
         </is>
       </c>
       <c r="E196" s="5" t="n">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="F196" s="9" t="n">
         <v>200</v>
@@ -7201,7 +7201,7 @@
         </is>
       </c>
       <c r="E197" s="5" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F197" s="9" t="n">
         <v>200</v>
@@ -7234,7 +7234,7 @@
         </is>
       </c>
       <c r="E198" s="5" t="n">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="F198" s="9" t="n">
         <v>200</v>
@@ -7267,7 +7267,7 @@
         </is>
       </c>
       <c r="E199" s="5" t="n">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="F199" s="9" t="n">
         <v>200</v>
@@ -7300,7 +7300,7 @@
         </is>
       </c>
       <c r="E200" s="5" t="n">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="F200" s="9" t="n">
         <v>200</v>
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="E201" s="5" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="F201" s="9" t="n">
         <v>200</v>
@@ -7366,7 +7366,7 @@
         </is>
       </c>
       <c r="E202" s="5" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="F202" s="9" t="n">
         <v>200</v>
@@ -7399,7 +7399,7 @@
         </is>
       </c>
       <c r="E203" s="5" t="n">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="F203" s="9" t="n">
         <v>200</v>
@@ -7432,7 +7432,7 @@
         </is>
       </c>
       <c r="E204" s="5" t="n">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F204" s="9" t="n">
         <v>200</v>
@@ -7465,7 +7465,7 @@
         </is>
       </c>
       <c r="E205" s="5" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F205" s="9" t="n">
         <v>200</v>
@@ -7498,7 +7498,7 @@
         </is>
       </c>
       <c r="E206" s="5" t="n">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="F206" s="9" t="n">
         <v>200</v>
@@ -7531,7 +7531,7 @@
         </is>
       </c>
       <c r="E207" s="5" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="F207" s="9" t="n">
         <v>200</v>
@@ -7564,7 +7564,7 @@
         </is>
       </c>
       <c r="E208" s="5" t="n">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="F208" s="9" t="n">
         <v>200</v>
@@ -7597,7 +7597,7 @@
         </is>
       </c>
       <c r="E209" s="5" t="n">
-        <v>95</v>
+        <v>36</v>
       </c>
       <c r="F209" s="9" t="n">
         <v>200</v>
@@ -7630,7 +7630,7 @@
         </is>
       </c>
       <c r="E210" s="5" t="n">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="F210" s="9" t="n">
         <v>200</v>
@@ -7663,7 +7663,7 @@
         </is>
       </c>
       <c r="E211" s="5" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F211" s="9" t="n">
         <v>200</v>
@@ -7696,7 +7696,7 @@
         </is>
       </c>
       <c r="E212" s="5" t="n">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="F212" s="9" t="n">
         <v>200</v>
@@ -7729,7 +7729,7 @@
         </is>
       </c>
       <c r="E213" s="5" t="n">
-        <v>17</v>
+        <v>74</v>
       </c>
       <c r="F213" s="9" t="n">
         <v>200</v>
@@ -7762,7 +7762,7 @@
         </is>
       </c>
       <c r="E214" s="5" t="n">
-        <v>56</v>
+        <v>92</v>
       </c>
       <c r="F214" s="9" t="n">
         <v>200</v>
@@ -7795,7 +7795,7 @@
         </is>
       </c>
       <c r="E215" s="5" t="n">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="F215" s="9" t="n">
         <v>200</v>
@@ -7828,7 +7828,7 @@
         </is>
       </c>
       <c r="E216" s="5" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F216" s="9" t="n">
         <v>200</v>
@@ -7861,7 +7861,7 @@
         </is>
       </c>
       <c r="E217" s="5" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="F217" s="9" t="n">
         <v>200</v>
@@ -7894,7 +7894,7 @@
         </is>
       </c>
       <c r="E218" s="5" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F218" s="9" t="n">
         <v>200</v>
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="E219" s="5" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="F219" s="9" t="n">
         <v>200</v>
@@ -7960,7 +7960,7 @@
         </is>
       </c>
       <c r="E220" s="5" t="n">
-        <v>69</v>
+        <v>15</v>
       </c>
       <c r="F220" s="9" t="n">
         <v>200</v>
@@ -7993,7 +7993,7 @@
         </is>
       </c>
       <c r="E221" s="5" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="F221" s="9" t="n">
         <v>200</v>
@@ -8026,7 +8026,7 @@
         </is>
       </c>
       <c r="E222" s="5" t="n">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="F222" s="9" t="n">
         <v>200</v>
@@ -8059,7 +8059,7 @@
         </is>
       </c>
       <c r="E223" s="5" t="n">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="F223" s="9" t="n">
         <v>200</v>
@@ -8092,7 +8092,7 @@
         </is>
       </c>
       <c r="E224" s="5" t="n">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="F224" s="9" t="n">
         <v>200</v>
@@ -8125,7 +8125,7 @@
         </is>
       </c>
       <c r="E225" s="5" t="n">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="F225" s="9" t="n">
         <v>200</v>
@@ -8158,7 +8158,7 @@
         </is>
       </c>
       <c r="E226" s="5" t="n">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="F226" s="9" t="n">
         <v>200</v>
@@ -8191,7 +8191,7 @@
         </is>
       </c>
       <c r="E227" s="5" t="n">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="F227" s="9" t="n">
         <v>200</v>
@@ -8224,7 +8224,7 @@
         </is>
       </c>
       <c r="E228" s="5" t="n">
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="F228" s="9" t="n">
         <v>200</v>
@@ -8257,7 +8257,7 @@
         </is>
       </c>
       <c r="E229" s="5" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F229" s="9" t="n">
         <v>200</v>
@@ -8290,7 +8290,7 @@
         </is>
       </c>
       <c r="E230" s="5" t="n">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="F230" s="9" t="n">
         <v>200</v>
@@ -8323,7 +8323,7 @@
         </is>
       </c>
       <c r="E231" s="5" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F231" s="9" t="n">
         <v>200</v>
@@ -8356,7 +8356,7 @@
         </is>
       </c>
       <c r="E232" s="5" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F232" s="9" t="n">
         <v>200</v>
@@ -8389,7 +8389,7 @@
         </is>
       </c>
       <c r="E233" s="5" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F233" s="9" t="n">
         <v>200</v>
@@ -8422,7 +8422,7 @@
         </is>
       </c>
       <c r="E234" s="5" t="n">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="F234" s="9" t="n">
         <v>200</v>
@@ -8455,7 +8455,7 @@
         </is>
       </c>
       <c r="E235" s="5" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="F235" s="9" t="n">
         <v>200</v>
@@ -8488,7 +8488,7 @@
         </is>
       </c>
       <c r="E236" s="5" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F236" s="9" t="n">
         <v>200</v>
@@ -8521,7 +8521,7 @@
         </is>
       </c>
       <c r="E237" s="5" t="n">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="F237" s="9" t="n">
         <v>200</v>
@@ -8554,7 +8554,7 @@
         </is>
       </c>
       <c r="E238" s="5" t="n">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="F238" s="9" t="n">
         <v>200</v>
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="E239" s="5" t="n">
-        <v>83</v>
+        <v>10</v>
       </c>
       <c r="F239" s="9" t="n">
         <v>200</v>
@@ -8620,7 +8620,7 @@
         </is>
       </c>
       <c r="E240" s="5" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F240" s="9" t="n">
         <v>200</v>
@@ -8653,7 +8653,7 @@
         </is>
       </c>
       <c r="E241" s="5" t="n">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="F241" s="9" t="n">
         <v>200</v>
@@ -8686,7 +8686,7 @@
         </is>
       </c>
       <c r="E242" s="5" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F242" s="9" t="n">
         <v>200</v>
@@ -8719,7 +8719,7 @@
         </is>
       </c>
       <c r="E243" s="5" t="n">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="F243" s="9" t="n">
         <v>200</v>
@@ -8752,7 +8752,7 @@
         </is>
       </c>
       <c r="E244" s="5" t="n">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="F244" s="9" t="n">
         <v>200</v>
@@ -8785,7 +8785,7 @@
         </is>
       </c>
       <c r="E245" s="5" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F245" s="9" t="n">
         <v>200</v>
@@ -8818,7 +8818,7 @@
         </is>
       </c>
       <c r="E246" s="5" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="F246" s="9" t="n">
         <v>200</v>
@@ -8851,7 +8851,7 @@
         </is>
       </c>
       <c r="E247" s="5" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="F247" s="9" t="n">
         <v>200</v>
@@ -8884,7 +8884,7 @@
         </is>
       </c>
       <c r="E248" s="5" t="n">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="F248" s="9" t="n">
         <v>200</v>
@@ -8917,7 +8917,7 @@
         </is>
       </c>
       <c r="E249" s="5" t="n">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="F249" s="9" t="n">
         <v>200</v>
@@ -8950,7 +8950,7 @@
         </is>
       </c>
       <c r="E250" s="5" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="F250" s="9" t="n">
         <v>200</v>
@@ -8983,7 +8983,7 @@
         </is>
       </c>
       <c r="E251" s="5" t="n">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="F251" s="9" t="n">
         <v>200</v>
@@ -9016,7 +9016,7 @@
         </is>
       </c>
       <c r="E252" s="5" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="F252" s="9" t="n">
         <v>200</v>
@@ -9049,7 +9049,7 @@
         </is>
       </c>
       <c r="E253" s="5" t="n">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="F253" s="9" t="n">
         <v>200</v>
@@ -9082,7 +9082,7 @@
         </is>
       </c>
       <c r="E254" s="5" t="n">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="F254" s="9" t="n">
         <v>200</v>
@@ -9115,7 +9115,7 @@
         </is>
       </c>
       <c r="E255" s="5" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F255" s="9" t="n">
         <v>200</v>
@@ -9148,7 +9148,7 @@
         </is>
       </c>
       <c r="E256" s="5" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="F256" s="9" t="n">
         <v>200</v>
@@ -9181,7 +9181,7 @@
         </is>
       </c>
       <c r="E257" s="5" t="n">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="F257" s="9" t="n">
         <v>200</v>
@@ -9214,7 +9214,7 @@
         </is>
       </c>
       <c r="E258" s="5" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F258" s="9" t="n">
         <v>200</v>
@@ -9247,7 +9247,7 @@
         </is>
       </c>
       <c r="E259" s="5" t="n">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="F259" s="9" t="n">
         <v>200</v>
@@ -9280,7 +9280,7 @@
         </is>
       </c>
       <c r="E260" s="5" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="F260" s="9" t="n">
         <v>200</v>
@@ -9313,7 +9313,7 @@
         </is>
       </c>
       <c r="E261" s="5" t="n">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="F261" s="9" t="n">
         <v>200</v>
@@ -9346,7 +9346,7 @@
         </is>
       </c>
       <c r="E262" s="5" t="n">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="F262" s="9" t="n">
         <v>200</v>
@@ -9379,7 +9379,7 @@
         </is>
       </c>
       <c r="E263" s="5" t="n">
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="F263" s="9" t="n">
         <v>200</v>
@@ -9412,7 +9412,7 @@
         </is>
       </c>
       <c r="E264" s="5" t="n">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="F264" s="9" t="n">
         <v>200</v>
@@ -9445,7 +9445,7 @@
         </is>
       </c>
       <c r="E265" s="5" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="F265" s="9" t="n">
         <v>200</v>
@@ -9478,7 +9478,7 @@
         </is>
       </c>
       <c r="E266" s="5" t="n">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="F266" s="9" t="n">
         <v>200</v>
@@ -9511,7 +9511,7 @@
         </is>
       </c>
       <c r="E267" s="5" t="n">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="F267" s="9" t="n">
         <v>200</v>
@@ -9544,7 +9544,7 @@
         </is>
       </c>
       <c r="E268" s="5" t="n">
-        <v>17</v>
+        <v>92</v>
       </c>
       <c r="F268" s="9" t="n">
         <v>200</v>
@@ -9610,7 +9610,7 @@
         </is>
       </c>
       <c r="E270" s="5" t="n">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="F270" s="9" t="n">
         <v>200</v>
@@ -9643,7 +9643,7 @@
         </is>
       </c>
       <c r="E271" s="5" t="n">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="F271" s="9" t="n">
         <v>200</v>
@@ -9676,7 +9676,7 @@
         </is>
       </c>
       <c r="E272" s="5" t="n">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="F272" s="9" t="n">
         <v>200</v>
@@ -9709,7 +9709,7 @@
         </is>
       </c>
       <c r="E273" s="5" t="n">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="F273" s="9" t="n">
         <v>200</v>
@@ -9742,7 +9742,7 @@
         </is>
       </c>
       <c r="E274" s="5" t="n">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="F274" s="9" t="n">
         <v>200</v>
@@ -9775,7 +9775,7 @@
         </is>
       </c>
       <c r="E275" s="5" t="n">
-        <v>76</v>
+        <v>32</v>
       </c>
       <c r="F275" s="9" t="n">
         <v>200</v>
@@ -9808,7 +9808,7 @@
         </is>
       </c>
       <c r="E276" s="5" t="n">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F276" s="9" t="n">
         <v>200</v>
@@ -9841,7 +9841,7 @@
         </is>
       </c>
       <c r="E277" s="5" t="n">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="F277" s="9" t="n">
         <v>200</v>
@@ -9874,7 +9874,7 @@
         </is>
       </c>
       <c r="E278" s="5" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="F278" s="9" t="n">
         <v>200</v>
@@ -9907,7 +9907,7 @@
         </is>
       </c>
       <c r="E279" s="5" t="n">
-        <v>44</v>
+        <v>94</v>
       </c>
       <c r="F279" s="9" t="n">
         <v>200</v>
@@ -9940,7 +9940,7 @@
         </is>
       </c>
       <c r="E280" s="5" t="n">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="F280" s="9" t="n">
         <v>200</v>
@@ -9973,7 +9973,7 @@
         </is>
       </c>
       <c r="E281" s="5" t="n">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="F281" s="9" t="n">
         <v>200</v>
@@ -10006,7 +10006,7 @@
         </is>
       </c>
       <c r="E282" s="5" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="F282" s="9" t="n">
         <v>200</v>
@@ -10039,7 +10039,7 @@
         </is>
       </c>
       <c r="E283" s="5" t="n">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="F283" s="9" t="n">
         <v>200</v>
@@ -10072,7 +10072,7 @@
         </is>
       </c>
       <c r="E284" s="5" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="F284" s="9" t="n">
         <v>200</v>
@@ -10105,7 +10105,7 @@
         </is>
       </c>
       <c r="E285" s="5" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="F285" s="9" t="n">
         <v>200</v>
@@ -10138,7 +10138,7 @@
         </is>
       </c>
       <c r="E286" s="5" t="n">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="F286" s="9" t="n">
         <v>200</v>
@@ -10171,7 +10171,7 @@
         </is>
       </c>
       <c r="E287" s="5" t="n">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="F287" s="9" t="n">
         <v>200</v>
@@ -10204,7 +10204,7 @@
         </is>
       </c>
       <c r="E288" s="5" t="n">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="F288" s="9" t="n">
         <v>200</v>
@@ -10237,7 +10237,7 @@
         </is>
       </c>
       <c r="E289" s="5" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F289" s="9" t="n">
         <v>200</v>
@@ -10270,7 +10270,7 @@
         </is>
       </c>
       <c r="E290" s="5" t="n">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="F290" s="9" t="n">
         <v>200</v>
@@ -10303,7 +10303,7 @@
         </is>
       </c>
       <c r="E291" s="5" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="F291" s="9" t="n">
         <v>200</v>
@@ -10336,7 +10336,7 @@
         </is>
       </c>
       <c r="E292" s="5" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F292" s="9" t="n">
         <v>200</v>
@@ -10369,7 +10369,7 @@
         </is>
       </c>
       <c r="E293" s="5" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="F293" s="9" t="n">
         <v>200</v>
@@ -10402,7 +10402,7 @@
         </is>
       </c>
       <c r="E294" s="5" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F294" s="9" t="n">
         <v>200</v>
@@ -10435,7 +10435,7 @@
         </is>
       </c>
       <c r="E295" s="5" t="n">
-        <v>15</v>
+        <v>68</v>
       </c>
       <c r="F295" s="9" t="n">
         <v>200</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="E296" s="5" t="n">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="F296" s="9" t="n">
         <v>200</v>
@@ -10501,7 +10501,7 @@
         </is>
       </c>
       <c r="E297" s="5" t="n">
-        <v>20</v>
+        <v>85</v>
       </c>
       <c r="F297" s="9" t="n">
         <v>200</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="E298" s="5" t="n">
-        <v>26</v>
+        <v>93</v>
       </c>
       <c r="F298" s="9" t="n">
         <v>200</v>
@@ -10567,7 +10567,7 @@
         </is>
       </c>
       <c r="E299" s="5" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="F299" s="9" t="n">
         <v>200</v>
@@ -10600,7 +10600,7 @@
         </is>
       </c>
       <c r="E300" s="5" t="n">
-        <v>19</v>
+        <v>68</v>
       </c>
       <c r="F300" s="9" t="n">
         <v>200</v>
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="E301" s="5" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F301" s="9" t="n">
         <v>200</v>

</xml_diff>